<commit_message>
chore: add latest comparison artifacts
</commit_message>
<xml_diff>
--- a/outputs/resultats/bns/2025_t2_vs_2025_t1/comparison.xlsx
+++ b/outputs/resultats/bns/2025_t2_vs_2025_t1/comparison.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Changements détectés" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Changements détectés'!$A$1:$N$15</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Changements détectés'!$A$1:$M$15</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -448,7 +448,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N15"/>
+  <dimension ref="A1:M15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -460,11 +460,10 @@
     <col width="50" customWidth="1" min="7" max="7"/>
     <col width="50" customWidth="1" min="8" max="8"/>
     <col width="70" customWidth="1" min="9" max="9"/>
-    <col width="22" customWidth="1" min="10" max="10"/>
+    <col width="16" customWidth="1" min="10" max="10"/>
     <col width="30" customWidth="1" min="11" max="11"/>
     <col width="16" customWidth="1" min="12" max="12"/>
-    <col width="18" customWidth="1" min="13" max="13"/>
-    <col width="22" customWidth="1" min="14" max="14"/>
+    <col width="22" customWidth="1" min="13" max="13"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -515,7 +514,7 @@
       </c>
       <c r="J1" s="1" t="inlineStr">
         <is>
-          <t>Nouvelle divulgation ?</t>
+          <t>Nouvelle idée ?</t>
         </is>
       </c>
       <c r="K1" s="1" t="inlineStr">
@@ -529,11 +528,6 @@
         </is>
       </c>
       <c r="M1" s="1" t="inlineStr">
-        <is>
-          <t>Validé par</t>
-        </is>
-      </c>
-      <c r="N1" s="1" t="inlineStr">
         <is>
           <t>Validé le</t>
         </is>
@@ -598,12 +592,7 @@
       </c>
       <c r="M2" s="2" t="inlineStr">
         <is>
-          <t>analyst</t>
-        </is>
-      </c>
-      <c r="N2" s="2" t="inlineStr">
-        <is>
-          <t>2026-04-19T00:08:32.496067+00:00</t>
+          <t>2026-05-15T01:19:05.653787+00:00</t>
         </is>
       </c>
     </row>
@@ -661,7 +650,6 @@
       <c r="K3" s="2" t="inlineStr"/>
       <c r="L3" s="2" t="inlineStr"/>
       <c r="M3" s="2" t="inlineStr"/>
-      <c r="N3" s="2" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -715,21 +703,8 @@
         </is>
       </c>
       <c r="K4" s="2" t="inlineStr"/>
-      <c r="L4" s="2" t="inlineStr">
-        <is>
-          <t>Validé</t>
-        </is>
-      </c>
-      <c r="M4" s="2" t="inlineStr">
-        <is>
-          <t>analyst</t>
-        </is>
-      </c>
-      <c r="N4" s="2" t="inlineStr">
-        <is>
-          <t>2026-04-19T00:08:33.686821+00:00</t>
-        </is>
-      </c>
+      <c r="L4" s="2" t="inlineStr"/>
+      <c r="M4" s="2" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -785,7 +760,6 @@
       <c r="K5" s="2" t="inlineStr"/>
       <c r="L5" s="2" t="inlineStr"/>
       <c r="M5" s="2" t="inlineStr"/>
-      <c r="N5" s="2" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -835,21 +809,8 @@
         </is>
       </c>
       <c r="K6" s="2" t="inlineStr"/>
-      <c r="L6" s="2" t="inlineStr">
-        <is>
-          <t>Validé</t>
-        </is>
-      </c>
-      <c r="M6" s="2" t="inlineStr">
-        <is>
-          <t>analyst</t>
-        </is>
-      </c>
-      <c r="N6" s="2" t="inlineStr">
-        <is>
-          <t>2026-04-19T00:08:27.047697+00:00</t>
-        </is>
-      </c>
+      <c r="L6" s="2" t="inlineStr"/>
+      <c r="M6" s="2" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
@@ -901,7 +862,6 @@
       <c r="K7" s="2" t="inlineStr"/>
       <c r="L7" s="2" t="inlineStr"/>
       <c r="M7" s="2" t="inlineStr"/>
-      <c r="N7" s="2" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
@@ -958,12 +918,7 @@
       </c>
       <c r="M8" s="2" t="inlineStr">
         <is>
-          <t>analyst</t>
-        </is>
-      </c>
-      <c r="N8" s="2" t="inlineStr">
-        <is>
-          <t>2026-04-19T00:08:36.126494+00:00</t>
+          <t>2026-05-15T01:19:20.610668+00:00</t>
         </is>
       </c>
     </row>
@@ -1015,21 +970,8 @@
         </is>
       </c>
       <c r="K9" s="2" t="inlineStr"/>
-      <c r="L9" s="2" t="inlineStr">
-        <is>
-          <t>Validé</t>
-        </is>
-      </c>
-      <c r="M9" s="2" t="inlineStr">
-        <is>
-          <t>analyst</t>
-        </is>
-      </c>
-      <c r="N9" s="2" t="inlineStr">
-        <is>
-          <t>2026-04-19T00:08:28.104931+00:00</t>
-        </is>
-      </c>
+      <c r="L9" s="2" t="inlineStr"/>
+      <c r="M9" s="2" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" s="3" t="inlineStr">
@@ -1086,12 +1028,7 @@
       </c>
       <c r="M10" s="3" t="inlineStr">
         <is>
-          <t>analyst</t>
-        </is>
-      </c>
-      <c r="N10" s="3" t="inlineStr">
-        <is>
-          <t>2026-04-19T00:07:59.165786+00:00</t>
+          <t>2026-05-15T01:18:51.064197+00:00</t>
         </is>
       </c>
     </row>
@@ -1150,12 +1087,7 @@
       </c>
       <c r="M11" s="3" t="inlineStr">
         <is>
-          <t>analyst</t>
-        </is>
-      </c>
-      <c r="N11" s="3" t="inlineStr">
-        <is>
-          <t>2026-04-19T00:07:59.323560+00:00</t>
+          <t>2026-05-15T01:18:51.419545+00:00</t>
         </is>
       </c>
     </row>
@@ -1207,21 +1139,8 @@
         </is>
       </c>
       <c r="K12" s="3" t="inlineStr"/>
-      <c r="L12" s="3" t="inlineStr">
-        <is>
-          <t>Validé</t>
-        </is>
-      </c>
-      <c r="M12" s="3" t="inlineStr">
-        <is>
-          <t>analyst</t>
-        </is>
-      </c>
-      <c r="N12" s="3" t="inlineStr">
-        <is>
-          <t>2026-04-19T00:08:31.167511+00:00</t>
-        </is>
-      </c>
+      <c r="L12" s="3" t="inlineStr"/>
+      <c r="M12" s="3" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" s="3" t="inlineStr">
@@ -1273,7 +1192,6 @@
       <c r="K13" s="3" t="inlineStr"/>
       <c r="L13" s="3" t="inlineStr"/>
       <c r="M13" s="3" t="inlineStr"/>
-      <c r="N13" s="3" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" s="3" t="inlineStr">
@@ -1325,7 +1243,6 @@
       <c r="K14" s="3" t="inlineStr"/>
       <c r="L14" s="3" t="inlineStr"/>
       <c r="M14" s="3" t="inlineStr"/>
-      <c r="N14" s="3" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" s="3" t="inlineStr">
@@ -1371,12 +1288,19 @@
         </is>
       </c>
       <c r="K15" s="3" t="inlineStr"/>
-      <c r="L15" s="3" t="inlineStr"/>
-      <c r="M15" s="3" t="inlineStr"/>
-      <c r="N15" s="3" t="inlineStr"/>
+      <c r="L15" s="3" t="inlineStr">
+        <is>
+          <t>Validé</t>
+        </is>
+      </c>
+      <c r="M15" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-15T01:19:46.877348+00:00</t>
+        </is>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:N15"/>
+  <autoFilter ref="A1:M15"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>